<commit_message>
site build 2026-10-08 21:21
</commit_message>
<xml_diff>
--- a/models/sovereigns/Ghana_Sovereign_Model.xlsx
+++ b/models/sovereigns/Ghana_Sovereign_Model.xlsx
@@ -700,7 +700,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Ghana Statistical Service, Consumer Price Index Bulletin Sep-26</t>
+          <t>Ghana Statistical Service, CPI Bulletin</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -739,11 +739,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -793,7 +789,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
+          <t>General government debt, IMF WEO</t>
         </is>
       </c>
     </row>
@@ -843,11 +839,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -929,11 +921,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1001,7 +989,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>BoG gross international reserves (approximate; gold inclusion not stated)</t>
+          <t>Bank of Ghana-reported gross; not reconciled with IMF International Liquidity gross incl. gold of 9.72 (Jul-26), 12.41 (Mar-26)</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1099,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>118.293</v>
+        <v>118.3</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1133,11 +1121,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1303,15 +1287,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>36-month non-financing Policy Coordination Instrument (PCI), following completion of the US$3.0B ECF</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>3</v>
+          <t>36-month non-financing Policy Coordination Instrument (PCI), following the US$3.0B ECF closed 27-Jul-26</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>27-Jul-26</t>
+        </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>15-Dec-26 first PCI monitoring mission</t>
+          <t>15-Dec-26 (first monitoring mission)</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1340,6 +1326,11 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Source</t>
         </is>
       </c>
@@ -1350,7 +1341,14 @@
           <t>nominal_gdp_usd_bn</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" s="2" t="n">
+        <v>118.3</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1358,7 +1356,14 @@
           <t>real_gdp_growth_pct</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1366,7 +1371,8 @@
           <t>cpi_avg_pct</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1374,7 +1380,14 @@
           <t>current_account_pct_gdp</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" s="2" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1382,7 +1395,14 @@
           <t>fiscal_balance_pct_gdp</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" s="2" t="n">
+        <v>-2.3</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1390,7 +1410,8 @@
           <t>primary_balance_pct_gdp</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1398,7 +1419,14 @@
           <t>gov_debt_pct_gdp</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1406,7 +1434,8 @@
           <t>external_debt_pct_gdp</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1414,7 +1443,8 @@
           <t>gross_reserves_usd_bn</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1422,7 +1452,8 @@
           <t>revenue_pct_gdp</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1430,7 +1461,8 @@
           <t>interest_pct_revenue</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
site build 2026-10-15 10:05
</commit_message>
<xml_diff>
--- a/models/sovereigns/Ghana_Sovereign_Model.xlsx
+++ b/models/sovereigns/Ghana_Sovereign_Model.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>as of 09-Oct-26</t>
+          <t>as of 15-Oct-26</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       <c r="D1" t="inlineStr"/>
       <c r="E1" t="inlineStr">
         <is>
-          <t>built 12-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/ghana.json</t>
+          <t>built 15-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/ghana.json</t>
         </is>
       </c>
     </row>
@@ -652,12 +652,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bank of Ghana, 132nd MPC Communiqué</t>
+          <t>Bank of Ghana MPC, via GNA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>28-Sep-26</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -700,12 +700,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Ghana Statistical Service CPI Bulletin</t>
+          <t>Ghana Statistical Service</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>07-Oct-26</t>
+          <t>15-Oct-26</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>4.8</v>
+        <v>6</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -726,17 +726,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026E</t>
+          <t>Q2-26</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
+          <t>Ghana Statistical Service via press</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>15-Oct-26</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -779,17 +779,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
+          <t>IMF WEO (database/sovereigns/ghana.json)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>09-Oct-26</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>IMF WEO general government debt</t>
+          <t>IMF WEO projection; press-quoted official figure of 45.9% (Dec-25: 44.7%) differs in definition and is unreconciled</t>
         </is>
       </c>
     </row>
@@ -831,12 +831,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
+          <t>IMF WEO (database/sovereigns/ghana.json)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>09-Oct-26</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -974,22 +974,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>end-Sep-26</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Bank of Ghana</t>
+          <t>Bank of Ghana via press</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>28-Sep-26</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>BoG-reported gross; definition not stated; not reconciled with IMF gross incl. gold of US$9.72B (Jul-26)</t>
+          <t>Bank of Ghana reported gross international reserves; unreconciled with IMF International Liquidity series (US$9.72bn incl. gold at Jul-26)</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>22-May-26</t>
+          <t>08-May-26</t>
         </is>
       </c>
     </row>
@@ -1253,7 +1253,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>18-Sep-26</t>
+          <t>27-Mar-26</t>
         </is>
       </c>
     </row>
@@ -1265,17 +1265,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Caa1</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Stable</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>16-Apr-26</t>
+          <t>09-Oct-26</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Policy Coordination Instrument (36-month, non-financing), following the completed US$3.0B ECF</t>
+          <t>36-month non-financing Policy Coordination Instrument (PCI), following completion of the 39-month US$3bn ECF on 27-Jul-26</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1297,7 +1297,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>15-Dec-26 (first monitoring mission)</t>
+          <t>15-Dec-26 (first PCI monitoring mission)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>moderate</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1366,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>IMF WEO, 08-Oct-26</t>
+          <t>IMF WEO, 09-Oct-26</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1405,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>IMF WEO, 08-Oct-26</t>
+          <t>IMF WEO, 09-Oct-26</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1429,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>IMF WEO, 08-Oct-26</t>
+          <t>IMF WEO, 09-Oct-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
site build 2026-10-23 10:05
</commit_message>
<xml_diff>
--- a/models/sovereigns/Ghana_Sovereign_Model.xlsx
+++ b/models/sovereigns/Ghana_Sovereign_Model.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>as of 15-Oct-26</t>
+          <t>as of 23-Oct-26</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       <c r="D1" t="inlineStr"/>
       <c r="E1" t="inlineStr">
         <is>
-          <t>built 19-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/ghana.json</t>
+          <t>built 23-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/ghana.json</t>
         </is>
       </c>
     </row>
@@ -652,12 +652,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bank of Ghana MPC, via GNA</t>
+          <t>Bank of Ghana MPC via GNA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>25-Sep-26</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -700,12 +700,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Ghana Statistical Service</t>
+          <t>GSS</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>15-Oct-26</t>
+          <t>23-Oct-26</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -731,12 +731,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Ghana Statistical Service via press</t>
+          <t>Press quoting GSS</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>15-Oct-26</t>
+          <t>23-Oct-26</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -774,22 +774,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026E</t>
+          <t>Jun-26</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>IMF WEO (database/sovereigns/ghana.json)</t>
+          <t>Ministry of Finance 2026 Mid-Year Budget Review via GNA</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>09-Oct-26</t>
+          <t>Jul-26</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>IMF WEO projection; press-quoted official figure of 45.9% (Dec-25: 44.7%) differs in definition and is unreconciled</t>
+          <t>Official government debt, mid-year budget review</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>-2.3</v>
+        <v>-0.4</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -826,17 +826,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026E</t>
+          <t>H1-26 (commitment basis; cash basis -0.8)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>IMF WEO (database/sovereigns/ghana.json)</t>
+          <t>Ministry of Finance 2026 Mid-Year Budget Review via GNA</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>09-Oct-26</t>
+          <t>Jul-26</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -864,15 +864,29 @@
           <t>interest_pct_revenue</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n"/>
+      <c r="B12" s="2" t="n">
+        <v>17.2</v>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>H1-26</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Moody's via MyJoyOnline</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>09-Oct-26</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -965,7 +979,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>12</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -974,22 +988,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>Jul-26</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Bank of Ghana via press</t>
+          <t>IMF International Liquidity</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>23-Oct-26</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Bank of Ghana reported gross international reserves; unreconciled with IMF International Liquidity series (US$9.72bn incl. gold at Jul-26)</t>
+          <t>gross incl. gold (IMF International Liquidity); BoG reports US$12.0bn at end-Sep-26 and US$12.9bn in Jun-26, unreconciled with the IMF series</t>
         </is>
       </c>
     </row>
@@ -1017,7 +1031,7 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>5.2</v>
+        <v>5</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1026,17 +1040,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>end-Sep-26</t>
+          <t>Jun-26</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Bank of Ghana</t>
+          <t>Bank of Ghana via press</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>28-Sep-26</t>
+          <t>23-Oct-26</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -1287,7 +1301,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>36-month non-financing Policy Coordination Instrument (PCI), following completion of the 39-month US$3bn ECF on 27-Jul-26</t>
+          <t>36-month non-financing Policy Coordination Instrument (PCI), following the US$3bn 39-month ECF completed 27-Jul-26</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1297,7 +1311,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>15-Dec-26 (first PCI monitoring mission)</t>
+          <t>15-Dec-26 (first monitoring mission under the PCI)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1317,7 +1331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1331,10 +1345,20 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>2026E</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -1346,10 +1370,12 @@
           <t>nominal_gdp_usd_bn</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n">
         <v>118.3</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>IMF WEO, 08-Oct-26</t>
         </is>
@@ -1361,12 +1387,14 @@
           <t>real_gdp_growth_pct</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n">
         <v>4.8</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>IMF WEO, 09-Oct-26</t>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>IMF WEO 2026E, as cited in reports/ghana-sovereign-credit.md, 23-Oct-26</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1405,9 @@
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1385,10 +1415,12 @@
           <t>current_account_pct_gdp</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n">
         <v>10.1</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>IMF WEO, 08-Oct-26</t>
         </is>
@@ -1400,12 +1432,14 @@
           <t>fiscal_balance_pct_gdp</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n">
         <v>-2.3</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>IMF WEO, 09-Oct-26</t>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>IMF WEO 2026E, as cited in reports/ghana-sovereign-credit.md, 23-Oct-26 (differs from the official commitment-basis figure; not reconciled)</t>
         </is>
       </c>
     </row>
@@ -1416,7 +1450,9 @@
         </is>
       </c>
       <c r="B7" s="2" t="n"/>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1425,11 +1461,17 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="D8" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>IMF WEO, 09-Oct-26</t>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Ministry of Finance 2026 Mid-Year Budget Review via GNA, Jul-26 (official definition; WEO 2026E of 53% not used because of the definition gap)</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1482,9 @@
         </is>
       </c>
       <c r="B9" s="2" t="n"/>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1449,7 +1493,9 @@
         </is>
       </c>
       <c r="B10" s="2" t="n"/>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1458,7 +1504,9 @@
         </is>
       </c>
       <c r="B11" s="2" t="n"/>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1467,7 +1515,9 @@
         </is>
       </c>
       <c r="B12" s="2" t="n"/>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>